<commit_message>
TamAssur facultatif pour les chauffeurs proprietaires (obligatoire en Cession), tricycle a 2 ans, plan et classeur recalcules
Proprietaires : adhesion et retrait depuis le tableau de bord, cotisation prelevee seulement apres adhesion, prelevement du 20 octobre rembourse, alerte de sortie pour restituer l'epargne. Tricycle : contrat de 24 mois (garantie TamAssur de 500 000 F a 24 mois = terme), assurance et tracker sans 2e anniversaire, cession au mois 25 dans le plan ; simulateur, CGU, guide et contrat (annexe 2) alignes. Test tamassur_optional_owner (8 controles).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TamCar_resultat_complet_v2.xlsx
+++ b/TamCar_resultat_complet_v2.xlsx
@@ -172,13 +172,13 @@
     <t>Seuils (taux d'atteinte minimal) :</t>
   </si>
   <si>
-    <t>excédent brut ≥ 0 aux années 2 et 3 : 98% ; résultat net ≥ 0 : 104% (après gadgets et gestes : 111%) ; caisse fin an 3 ≥ 0 : 75%</t>
+    <t>excédent brut ≥ 0 aux années 2 et 3 : 103% ; résultat net ≥ 0 : 106% (après gadgets et gestes : 113%) ; caisse fin an 3 ≥ 0 : 76%</t>
   </si>
   <si>
     <t>B. Avec le minimum décidé : 3 Essentiel + 3 Confort de tiers, arrivées étalées du mois 4 au mois 12</t>
   </si>
   <si>
-    <t>excédent brut ≥ 0 aux années 2 et 3 : 76% ; résultat net ≥ 0 : 80% (après gadgets et gestes : 84%) ; caisse fin an 3 ≥ 0 : 64%</t>
+    <t>excédent brut ≥ 0 aux années 2 et 3 : 78% ; résultat net ≥ 0 : 79% (après gadgets et gestes : 83%) ; caisse fin an 3 ≥ 0 : 64%</t>
   </si>
   <si>
     <t>C. Valeur mensuelle nette d'un véhicule de tiers en régime établi (après part du responsable des opérations et postes vacants), FCFA par mois</t>
@@ -739,7 +739,7 @@
     <t>Durée avant cession du tricycle (mois)</t>
   </si>
   <si>
-    <t>Plan d'affaires : 36 mois ; le fonds de rachat est encaissé à la cession, hors des 36 mois affichés</t>
+    <t>Terence (2026-10-21) : 2 ans pour le tricycle (garantie TamAssur de 500 000 F à 24 mois, qui est aussi le terme) ; assurance et tracker payés à l'achat puis au 1er anniversaire seulement ; 20 % de commission ensuite</t>
   </si>
   <si>
     <t>Objectif du jour d'une moto de TamCar, tout compris (versement 2 500 F + TamAssur 1 000 F)</t>
@@ -2185,11 +2185,11 @@
       </c>
       <c r="D6" s="24">
         <f>Résultat!D6</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
       <c r="E6" s="24">
         <f>Résultat!E6</f>
-        <v>46226375</v>
+        <v>45446375</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -2206,11 +2206,11 @@
       </c>
       <c r="D7" s="22">
         <f>Résultat!D7+Résultat!D8</f>
-        <v>-10948250</v>
+        <v>-10784250</v>
       </c>
       <c r="E7" s="22">
         <f>Résultat!E7+Résultat!E8</f>
-        <v>-31389611</v>
+        <v>-31225611</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -2227,11 +2227,11 @@
       </c>
       <c r="D8" s="24">
         <f>Résultat!D9</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E8" s="24">
         <f>Résultat!E9</f>
-        <v>14836764</v>
+        <v>14220764</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -2240,15 +2240,15 @@
       </c>
       <c r="B9" s="22">
         <f>Résultat!B10+Résultat!B11</f>
-        <v>-6275000</v>
+        <v>-6533333.333333334</v>
       </c>
       <c r="C9" s="22">
         <f>Résultat!C10+Résultat!C11</f>
-        <v>-850000.00000000012</v>
+        <v>-1108333.3333333333</v>
       </c>
       <c r="D9" s="22">
         <f>Résultat!D10+Résultat!D11</f>
-        <v>-850000.00000000012</v>
+        <v>-333333.33333333326</v>
       </c>
       <c r="E9" s="22">
         <f>Résultat!E10+Résultat!E11</f>
@@ -2261,19 +2261,19 @@
       </c>
       <c r="B10" s="24">
         <f>Résultat!B14</f>
-        <v>-2129136</v>
+        <v>-2387469.333333334</v>
       </c>
       <c r="C10" s="24">
         <f>Résultat!C14</f>
-        <v>4806950</v>
+        <v>4548616.666666667</v>
       </c>
       <c r="D10" s="24">
         <f>Résultat!D14</f>
-        <v>2928765</v>
+        <v>2859231.666666667</v>
       </c>
       <c r="E10" s="24">
         <f>Résultat!E14</f>
-        <v>5606579</v>
+        <v>5020379</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -2303,19 +2303,19 @@
       </c>
       <c r="B12" s="24">
         <f>Résultat!B19</f>
-        <v>-2824136</v>
+        <v>-3082469.333333334</v>
       </c>
       <c r="C12" s="24">
         <f>Résultat!C19</f>
-        <v>4016950</v>
+        <v>3758616.666666667</v>
       </c>
       <c r="D12" s="24">
         <f>Résultat!D19</f>
-        <v>2138765</v>
+        <v>2069231.666666667</v>
       </c>
       <c r="E12" s="24">
         <f>Résultat!E19</f>
-        <v>3331579</v>
+        <v>2745379</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -2332,11 +2332,11 @@
       </c>
       <c r="D13" s="22">
         <f>Résultat!D31</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E13" s="22">
         <f>Résultat!E31</f>
-        <v>6361764.0000000009</v>
+        <v>5745764.0000000009</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="D14" s="24">
         <f>Résultat!D33</f>
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
       <c r="E14" s="10"/>
     </row>
@@ -2371,11 +2371,11 @@
       </c>
       <c r="D15" s="36">
         <f>IF(D6=0,0,D8/D6)</f>
-        <v>0.31497228166335045</v>
+        <v>0.29061254292141925</v>
       </c>
       <c r="E15" s="36">
         <f>IF(E6=0,0,E8/E6)</f>
-        <v>0.32095884654593831</v>
+        <v>0.31291305412147835</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -2435,15 +2435,15 @@
       </c>
       <c r="C20" s="22">
         <f>Marge!C11</f>
-        <v>531101.35670502495</v>
+        <v>272768.02337169158</v>
       </c>
       <c r="D20" s="36">
         <f>Marge!C12</f>
-        <v>0.3947241595726681</v>
+        <v>0.2027261414876935</v>
       </c>
       <c r="E20" s="22">
         <f>Marge!C14</f>
-        <v>-150223.13113764767</v>
+        <v>-408556.46447098104</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -2498,15 +2498,15 @@
       </c>
       <c r="C23" s="24">
         <f>Marge!F11</f>
-        <v>8476072.333333334</v>
+        <v>8217739</v>
       </c>
       <c r="D23" s="37">
         <f>Marge!F12</f>
-        <v>0.59431266240007674</v>
+        <v>0.57619922906890531</v>
       </c>
       <c r="E23" s="24">
         <f>Marge!F14</f>
-        <v>1254197.333333334</v>
+        <v>995864</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -8282,158 +8282,158 @@
       </c>
       <c r="E48" s="22">
         <f>SUM(AF48:AQ48)</f>
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="F48" s="22">
         <f>SUM(B48:E48)</f>
-        <v>225000</v>
+        <v>150000</v>
       </c>
       <c r="G48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=G$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=G$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=G$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=G$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=G$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="H48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=H$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=H$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=H$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=H$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=H$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>75000</v>
       </c>
       <c r="I48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=I$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=I$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=I$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=I$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=I$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="J48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=J$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=J$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=J$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=J$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=J$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="K48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=K$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=K$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=K$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=K$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=K$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="L48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=L$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=L$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=L$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=L$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=L$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="M48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=M$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=M$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=M$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=M$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=M$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="N48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=N$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=N$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=N$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=N$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=N$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="O48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=O$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=O$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=O$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=O$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=O$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="P48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=P$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=P$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=P$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=P$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=P$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="Q48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=Q$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Q$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Q$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=Q$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Q$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="R48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=R$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=R$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=R$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=R$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=R$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="S48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=S$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=S$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=S$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=S$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=S$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="T48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=T$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=T$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=T$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=T$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=T$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>75000</v>
       </c>
       <c r="U48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=U$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=U$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=U$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=U$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=U$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="V48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=V$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=V$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=V$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=V$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=V$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="W48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=W$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=W$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=W$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=W$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=W$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="X48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=X$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=X$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=X$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=X$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=X$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="Y48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=Y$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Y$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Y$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=Y$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Y$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="Z48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=Z$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Z$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Z$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=Z$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Z$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AA48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AA$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AA$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AA$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AA$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AA$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AB48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AB$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AB$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AB$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AB$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AB$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AC48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AC$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AC$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AC$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AC$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AC$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AD48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AD$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AD$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AD$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AD$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AD$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AE48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AE$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AE$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AE$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AE$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AE$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AF48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AF$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AF$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AF$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
-        <v>75000</v>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AF$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AF$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <v>0</v>
       </c>
       <c r="AG48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AG$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AG$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AG$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AG$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AG$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AH48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AH$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AH$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AH$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AH$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AH$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AI48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AI$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AI$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AI$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AI$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AI$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AJ48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AJ$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AJ$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AJ$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AJ$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AJ$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AK48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AK$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AK$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AK$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AK$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AK$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AL48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AL$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AL$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AL$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AL$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AL$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AM48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AM$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AM$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AM$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AM$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AM$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AN48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AN$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AN$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AN$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AN$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AN$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AO48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AO$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AO$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AO$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AO$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AO$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AP48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AP$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AP$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AP$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AP$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AP$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
       <c r="AQ48" s="22">
-        <f>(SUMPRODUCT(($G$4:$AQ$4=AQ$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AQ$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AQ$4-24)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
+        <f>(SUMPRODUCT(($G$4:$AQ$4=AQ$4)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AQ$4-12)*$G$7:$AQ$7))*Hypothèses!$B$15</f>
         <v>0</v>
       </c>
     </row>
@@ -8628,158 +8628,158 @@
       </c>
       <c r="E50" s="22">
         <f>SUM(AF50:AQ50)</f>
-        <v>89000</v>
+        <v>0</v>
       </c>
       <c r="F50" s="22">
         <f>SUM(B50:E50)</f>
-        <v>317000</v>
+        <v>228000</v>
       </c>
       <c r="G50" s="22">
-        <f>G7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=G$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=G$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>G7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=G$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="H50" s="22">
-        <f>H7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=H$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=H$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>H7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=H$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>139000</v>
       </c>
       <c r="I50" s="22">
-        <f>I7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=I$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=I$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>I7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=I$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="J50" s="22">
-        <f>J7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=J$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=J$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>J7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=J$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="K50" s="22">
-        <f>K7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=K$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=K$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>K7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=K$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="L50" s="22">
-        <f>L7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=L$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=L$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>L7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=L$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="M50" s="22">
-        <f>M7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=M$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=M$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>M7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=M$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="N50" s="22">
-        <f>N7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=N$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=N$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>N7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=N$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="O50" s="22">
-        <f>O7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=O$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=O$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>O7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=O$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="P50" s="22">
-        <f>P7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=P$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=P$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>P7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=P$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="Q50" s="22">
-        <f>Q7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Q$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Q$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>Q7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Q$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="R50" s="22">
-        <f>R7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=R$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=R$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>R7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=R$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="S50" s="22">
-        <f>S7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=S$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=S$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>S7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=S$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="T50" s="22">
-        <f>T7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=T$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=T$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>T7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=T$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>89000</v>
       </c>
       <c r="U50" s="22">
-        <f>U7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=U$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=U$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>U7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=U$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="V50" s="22">
-        <f>V7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=V$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=V$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>V7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=V$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="W50" s="22">
-        <f>W7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=W$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=W$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>W7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=W$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="X50" s="22">
-        <f>X7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=X$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=X$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>X7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=X$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="Y50" s="22">
-        <f>Y7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Y$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Y$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>Y7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Y$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="Z50" s="22">
-        <f>Z7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Z$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=Z$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>Z7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=Z$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AA50" s="22">
-        <f>AA7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AA$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AA$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AA7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AA$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AB50" s="22">
-        <f>AB7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AB$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AB$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AB7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AB$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AC50" s="22">
-        <f>AC7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AC$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AC$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AC7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AC$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AD50" s="22">
-        <f>AD7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AD$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AD$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AD7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AD$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AE50" s="22">
-        <f>AE7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AE$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AE$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AE7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AE$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AF50" s="22">
-        <f>AF7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AF$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AF$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
-        <v>89000</v>
+        <f>AF7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AF$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <v>0</v>
       </c>
       <c r="AG50" s="22">
-        <f>AG7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AG$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AG$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AG7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AG$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AH50" s="22">
-        <f>AH7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AH$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AH$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AH7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AH$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AI50" s="22">
-        <f>AI7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AI$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AI$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AI7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AI$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AJ50" s="22">
-        <f>AJ7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AJ$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AJ$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AJ7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AJ$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AK50" s="22">
-        <f>AK7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AK$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AK$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AK7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AK$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AL50" s="22">
-        <f>AL7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AL$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AL$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AL7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AL$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AM50" s="22">
-        <f>AM7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AM$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AM$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AM7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AM$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AN50" s="22">
-        <f>AN7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AN$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AN$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AN7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AN$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AO50" s="22">
-        <f>AO7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AO$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AO$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AO7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AO$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AP50" s="22">
-        <f>AP7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AP$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AP$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AP7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AP$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
       <c r="AQ50" s="22">
-        <f>AQ7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AQ$4-12)*$G$7:$AQ$7)+SUMPRODUCT(($G$4:$AQ$4=AQ$4-24)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
+        <f>AQ7*Hypothèses!$B$17+(SUMPRODUCT(($G$4:$AQ$4=AQ$4-12)*$G$7:$AQ$7))*Hypothèses!$B$18</f>
         <v>0</v>
       </c>
     </row>
@@ -8974,11 +8974,11 @@
       </c>
       <c r="E52" s="23">
         <f>SUM(AF52:AQ52)</f>
-        <v>164000</v>
+        <v>0</v>
       </c>
       <c r="F52" s="23">
         <f>SUM(B52:E52)</f>
-        <v>1487000</v>
+        <v>1323000</v>
       </c>
       <c r="G52" s="23">
         <f t="shared" ref="G52:AQ52" si="15">SUM(G48:G51)</f>
@@ -9082,7 +9082,7 @@
       </c>
       <c r="AF52" s="23">
         <f t="shared" si="15"/>
-        <v>164000</v>
+        <v>0</v>
       </c>
       <c r="AG52" s="23">
         <f t="shared" si="15"/>
@@ -9147,11 +9147,11 @@
       </c>
       <c r="E54" s="24">
         <f>SUM(AF54:AQ54)</f>
-        <v>10948250</v>
+        <v>10784250</v>
       </c>
       <c r="F54" s="24">
         <f>SUM(B54:E54)</f>
-        <v>39864611</v>
+        <v>39700611</v>
       </c>
       <c r="G54" s="24">
         <f t="shared" ref="G54:AQ54" si="16">G20+G39+G45+G52</f>
@@ -9255,7 +9255,7 @@
       </c>
       <c r="AF54" s="24">
         <f t="shared" si="16"/>
-        <v>1830187.5</v>
+        <v>1666187.5</v>
       </c>
       <c r="AG54" s="24">
         <f t="shared" si="16"/>
@@ -9408,51 +9408,51 @@
       </c>
       <c r="AF55" s="25">
         <f t="shared" si="17"/>
-        <v>30746548.5</v>
+        <v>30582548.5</v>
       </c>
       <c r="AG55" s="25">
         <f t="shared" si="17"/>
-        <v>31480736</v>
+        <v>31316736</v>
       </c>
       <c r="AH55" s="25">
         <f t="shared" si="17"/>
-        <v>32339923.5</v>
+        <v>32175923.5</v>
       </c>
       <c r="AI55" s="25">
         <f t="shared" si="17"/>
-        <v>33328111</v>
+        <v>33164111</v>
       </c>
       <c r="AJ55" s="25">
         <f t="shared" si="17"/>
-        <v>34158298.5</v>
+        <v>33994298.5</v>
       </c>
       <c r="AK55" s="25">
         <f t="shared" si="17"/>
-        <v>35017486</v>
+        <v>34853486</v>
       </c>
       <c r="AL55" s="25">
         <f t="shared" si="17"/>
-        <v>35751673.5</v>
+        <v>35587673.5</v>
       </c>
       <c r="AM55" s="25">
         <f t="shared" si="17"/>
-        <v>36581861</v>
+        <v>36417861</v>
       </c>
       <c r="AN55" s="25">
         <f t="shared" si="17"/>
-        <v>37441048.5</v>
+        <v>37277048.5</v>
       </c>
       <c r="AO55" s="25">
         <f t="shared" si="17"/>
-        <v>38175236</v>
+        <v>38011236</v>
       </c>
       <c r="AP55" s="25">
         <f t="shared" si="17"/>
-        <v>39005423.5</v>
+        <v>38841423.5</v>
       </c>
       <c r="AQ55" s="25">
         <f t="shared" si="17"/>
-        <v>39864611</v>
+        <v>39700611</v>
       </c>
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.3">
@@ -9520,11 +9520,11 @@
       </c>
       <c r="E58" s="22">
         <f>SUM(AF58:AQ58)</f>
-        <v>1404000</v>
+        <v>624000</v>
       </c>
       <c r="F58" s="22">
         <f>SUM(B58:E58)</f>
-        <v>4153500</v>
+        <v>3373500</v>
       </c>
       <c r="G58" s="22">
         <v>0</v>
@@ -9627,51 +9627,51 @@
       </c>
       <c r="AF58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AF$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AF$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AF$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AF$4-$G$4:$AQ$4)&gt;=12)*((AF$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AF$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AF94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AF98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AG58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AG$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AG$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AG$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AG$4-$G$4:$AQ$4)&gt;=12)*((AG$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AG$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AG94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AG98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AH58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AH$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AH$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AH$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AH$4-$G$4:$AQ$4)&gt;=12)*((AH$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AH$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AH94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AH98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AI58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AI$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AI$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AI$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AI$4-$G$4:$AQ$4)&gt;=12)*((AI$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AI$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AI94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AI98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AJ58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AJ$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AJ$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AJ$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AJ$4-$G$4:$AQ$4)&gt;=12)*((AJ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AJ$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AJ94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AJ98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AK58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AK$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AK$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AK$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AK$4-$G$4:$AQ$4)&gt;=12)*((AK$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AK$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AK94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AK98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AL58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AL$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AL$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AL$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AL$4-$G$4:$AQ$4)&gt;=12)*((AL$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AL$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AL94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AL98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AM58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AM$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AM$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AM$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AM$4-$G$4:$AQ$4)&gt;=12)*((AM$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AM$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AM94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AM98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AN58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AN$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AN$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AN$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AN$4-$G$4:$AQ$4)&gt;=12)*((AN$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AN$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AN94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AN98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AO58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AO$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AO$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AO$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AO$4-$G$4:$AQ$4)&gt;=12)*((AO$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AO$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AO94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AO98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AP58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AP$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AP$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AP$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AP$4-$G$4:$AQ$4)&gt;=12)*((AP$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AP$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AP94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AP98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
       <c r="AQ58" s="22">
         <f>(Hypothèses!$B$45*Hypothèses!$B$47*SUMPRODUCT($G$7:$AQ$7*((AQ$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AQ$4-$G$4:$AQ$4)=0))*(Hypothèses!$B$71*((AQ$4-$G$4:$AQ$4)&lt;12)+Hypothèses!$B$72*((AQ$4-$G$4:$AQ$4)&gt;=12)*((AQ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74)+Hypothèses!$B$73*((AQ$4-$G$4:$AQ$4)&gt;=Hypothèses!$B$74))))*Hypothèses!$B$94+AQ94*Hypothèses!$B$102-Hypothèses!$B$103*Hypothèses!$B$47*AQ98</f>
-        <v>117000</v>
+        <v>52000</v>
       </c>
     </row>
     <row r="59" spans="1:43" x14ac:dyDescent="0.3">
@@ -10208,11 +10208,11 @@
       </c>
       <c r="E62" s="24">
         <f>SUM(AF62:AQ62)</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
       <c r="F62" s="24">
         <f>SUM(B62:E62)</f>
-        <v>46226375</v>
+        <v>45446375</v>
       </c>
       <c r="G62" s="24">
         <f t="shared" ref="G62:AQ62" si="18">SUM(G58:G61)</f>
@@ -10316,51 +10316,51 @@
       </c>
       <c r="AF62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AG62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AH62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AI62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AJ62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AK62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AL62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AM62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AN62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AO62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AP62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
       <c r="AQ62" s="24">
         <f t="shared" si="18"/>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
     </row>
     <row r="64" spans="1:43" x14ac:dyDescent="0.3">
@@ -10428,11 +10428,11 @@
       </c>
       <c r="E65" s="25">
         <f>SUM(AF65:AQ65)</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="F65" s="25">
         <f>SUM(B65:E65)</f>
-        <v>6361764.0000000009</v>
+        <v>5745764.0000000009</v>
       </c>
       <c r="G65" s="25">
         <f t="shared" ref="G65:AQ65" si="19">G62-G54</f>
@@ -10536,51 +10536,51 @@
       </c>
       <c r="AF65" s="25">
         <f t="shared" si="19"/>
-        <v>-498337.5</v>
+        <v>-399337.5</v>
       </c>
       <c r="AG65" s="25">
         <f t="shared" si="19"/>
-        <v>597662.5</v>
+        <v>532662.5</v>
       </c>
       <c r="AH65" s="25">
         <f t="shared" si="19"/>
-        <v>472662.5</v>
+        <v>407662.5</v>
       </c>
       <c r="AI65" s="25">
         <f t="shared" si="19"/>
-        <v>343662.5</v>
+        <v>278662.5</v>
       </c>
       <c r="AJ65" s="25">
         <f t="shared" si="19"/>
-        <v>501662.5</v>
+        <v>436662.5</v>
       </c>
       <c r="AK65" s="25">
         <f t="shared" si="19"/>
-        <v>472662.5</v>
+        <v>407662.5</v>
       </c>
       <c r="AL65" s="25">
         <f t="shared" si="19"/>
-        <v>597662.5</v>
+        <v>532662.5</v>
       </c>
       <c r="AM65" s="25">
         <f t="shared" si="19"/>
-        <v>501662.5</v>
+        <v>436662.5</v>
       </c>
       <c r="AN65" s="25">
         <f t="shared" si="19"/>
-        <v>472662.5</v>
+        <v>407662.5</v>
       </c>
       <c r="AO65" s="25">
         <f t="shared" si="19"/>
-        <v>597662.5</v>
+        <v>532662.5</v>
       </c>
       <c r="AP65" s="25">
         <f t="shared" si="19"/>
-        <v>501662.5</v>
+        <v>436662.5</v>
       </c>
       <c r="AQ65" s="25">
         <f t="shared" si="19"/>
-        <v>472662.5</v>
+        <v>407662.5</v>
       </c>
     </row>
     <row r="66" spans="1:43" x14ac:dyDescent="0.3">
@@ -10601,7 +10601,7 @@
       </c>
       <c r="E66" s="24">
         <f>AQ66</f>
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
       <c r="F66" s="24">
         <f>MIN(G66:AQ66)</f>
@@ -10709,51 +10709,51 @@
       </c>
       <c r="AF66" s="24">
         <f t="shared" si="20"/>
-        <v>15829476.5</v>
+        <v>15928476.5</v>
       </c>
       <c r="AG66" s="24">
         <f t="shared" si="20"/>
-        <v>16427139</v>
+        <v>16461139</v>
       </c>
       <c r="AH66" s="24">
         <f t="shared" si="20"/>
-        <v>16899801.5</v>
+        <v>16868801.5</v>
       </c>
       <c r="AI66" s="24">
         <f t="shared" si="20"/>
-        <v>17243464</v>
+        <v>17147464</v>
       </c>
       <c r="AJ66" s="24">
         <f t="shared" si="20"/>
-        <v>17745126.5</v>
+        <v>17584126.5</v>
       </c>
       <c r="AK66" s="24">
         <f t="shared" si="20"/>
-        <v>18217789</v>
+        <v>17991789</v>
       </c>
       <c r="AL66" s="24">
         <f t="shared" si="20"/>
-        <v>18815451.5</v>
+        <v>18524451.5</v>
       </c>
       <c r="AM66" s="24">
         <f t="shared" si="20"/>
-        <v>19317114</v>
+        <v>18961114</v>
       </c>
       <c r="AN66" s="24">
         <f t="shared" si="20"/>
-        <v>19789776.5</v>
+        <v>19368776.5</v>
       </c>
       <c r="AO66" s="24">
         <f t="shared" si="20"/>
-        <v>20387439</v>
+        <v>19901439</v>
       </c>
       <c r="AP66" s="24">
         <f t="shared" si="20"/>
-        <v>20889101.5</v>
+        <v>20338101.5</v>
       </c>
       <c r="AQ66" s="24">
         <f t="shared" si="20"/>
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
     </row>
     <row r="67" spans="1:43" x14ac:dyDescent="0.3">
@@ -10973,19 +10973,19 @@
       </c>
       <c r="C70" s="22">
         <f t="shared" ref="C70:C77" si="23">SUM(H70:S70)</f>
-        <v>516666.66666666669</v>
+        <v>775000.00000000012</v>
       </c>
       <c r="D70" s="22">
         <f t="shared" ref="D70:D77" si="24">SUM(T70:AE70)</f>
-        <v>516666.66666666669</v>
+        <v>775000.00000000012</v>
       </c>
       <c r="E70" s="22">
         <f t="shared" ref="E70:E77" si="25">SUM(AF70:AQ70)</f>
-        <v>516666.66666666669</v>
+        <v>0</v>
       </c>
       <c r="F70" s="22">
         <f t="shared" ref="F70:F77" si="26">SUM(B70:E70)</f>
-        <v>1550000</v>
+        <v>1550000.0000000002</v>
       </c>
       <c r="G70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((G$4-$G$4:$AQ$4)&gt;=0)*((G$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
@@ -10993,147 +10993,147 @@
       </c>
       <c r="H70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((H$4-$G$4:$AQ$4)&gt;=0)*((H$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="I70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((I$4-$G$4:$AQ$4)&gt;=0)*((I$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="J70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((J$4-$G$4:$AQ$4)&gt;=0)*((J$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="K70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((K$4-$G$4:$AQ$4)&gt;=0)*((K$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="L70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((L$4-$G$4:$AQ$4)&gt;=0)*((L$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="M70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((M$4-$G$4:$AQ$4)&gt;=0)*((M$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="N70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((N$4-$G$4:$AQ$4)&gt;=0)*((N$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="O70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((O$4-$G$4:$AQ$4)&gt;=0)*((O$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="P70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((P$4-$G$4:$AQ$4)&gt;=0)*((P$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="Q70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((Q$4-$G$4:$AQ$4)&gt;=0)*((Q$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="R70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((R$4-$G$4:$AQ$4)&gt;=0)*((R$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="S70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((S$4-$G$4:$AQ$4)&gt;=0)*((S$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="T70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((T$4-$G$4:$AQ$4)&gt;=0)*((T$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="U70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((U$4-$G$4:$AQ$4)&gt;=0)*((U$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="V70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((V$4-$G$4:$AQ$4)&gt;=0)*((V$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="W70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((W$4-$G$4:$AQ$4)&gt;=0)*((W$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="X70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((X$4-$G$4:$AQ$4)&gt;=0)*((X$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="Y70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((Y$4-$G$4:$AQ$4)&gt;=0)*((Y$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="Z70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((Z$4-$G$4:$AQ$4)&gt;=0)*((Z$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AA70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AA$4-$G$4:$AQ$4)&gt;=0)*((AA$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AB70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AB$4-$G$4:$AQ$4)&gt;=0)*((AB$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AC70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AC$4-$G$4:$AQ$4)&gt;=0)*((AC$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AD70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AD$4-$G$4:$AQ$4)&gt;=0)*((AD$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AE70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AE$4-$G$4:$AQ$4)&gt;=0)*((AE$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>64583.333333333336</v>
       </c>
       <c r="AF70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AF$4-$G$4:$AQ$4)&gt;=0)*((AF$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AG70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AG$4-$G$4:$AQ$4)&gt;=0)*((AG$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AH70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AH$4-$G$4:$AQ$4)&gt;=0)*((AH$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AI70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AI$4-$G$4:$AQ$4)&gt;=0)*((AI$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AJ70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AJ$4-$G$4:$AQ$4)&gt;=0)*((AJ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AK70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AK$4-$G$4:$AQ$4)&gt;=0)*((AK$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AL70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AL$4-$G$4:$AQ$4)&gt;=0)*((AL$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AM70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AM$4-$G$4:$AQ$4)&gt;=0)*((AM$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AN70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AN$4-$G$4:$AQ$4)&gt;=0)*((AN$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AO70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AO$4-$G$4:$AQ$4)&gt;=0)*((AO$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AP70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AP$4-$G$4:$AQ$4)&gt;=0)*((AP$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
       <c r="AQ70" s="22">
         <f>SUMPRODUCT($G$7:$AQ$7*((AQ$4-$G$4:$AQ$4)&gt;=0)*((AQ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))*Hypothèses!$B$9/Hypothèses!$B$74</f>
-        <v>43055.555555555555</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:43" x14ac:dyDescent="0.3">
@@ -11492,15 +11492,15 @@
       </c>
       <c r="C73" s="24">
         <f t="shared" si="23"/>
-        <v>3225000</v>
+        <v>3483333.333333334</v>
       </c>
       <c r="D73" s="24">
         <f t="shared" si="24"/>
-        <v>850000.00000000012</v>
+        <v>1108333.3333333333</v>
       </c>
       <c r="E73" s="24">
         <f t="shared" si="25"/>
-        <v>850000.00000000012</v>
+        <v>333333.33333333326</v>
       </c>
       <c r="F73" s="24">
         <f t="shared" si="26"/>
@@ -11512,147 +11512,147 @@
       </c>
       <c r="H73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="I73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="J73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="K73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="L73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="M73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="N73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="O73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="P73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="Q73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="R73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="S73" s="24">
         <f t="shared" si="27"/>
-        <v>268750</v>
+        <v>290277.77777777775</v>
       </c>
       <c r="T73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="U73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="V73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="W73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="X73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="Y73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="Z73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AA73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AB73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AC73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AD73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AE73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>92361.111111111109</v>
       </c>
       <c r="AF73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AG73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AH73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AI73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AJ73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AK73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AL73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AM73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AN73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AO73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AP73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
       <c r="AQ73" s="24">
         <f t="shared" si="27"/>
-        <v>70833.333333333328</v>
+        <v>27777.777777777777</v>
       </c>
     </row>
     <row r="74" spans="1:43" x14ac:dyDescent="0.3">
@@ -15101,11 +15101,11 @@
       </c>
       <c r="E98" s="22">
         <f t="shared" ref="E98:E105" si="39">SUM(AF98:AQ98)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F98" s="22">
         <f t="shared" ref="F98:F105" si="40">SUM(B98:E98)</f>
-        <v>35.5</v>
+        <v>23.5</v>
       </c>
       <c r="G98" s="39">
         <f>0</f>
@@ -15209,51 +15209,51 @@
       </c>
       <c r="AF98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AF$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AF$4-$G$4:$AQ$4)=0))*((AF$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AF89-0.5*(AF89-AE89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AG$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AG$4-$G$4:$AQ$4)=0))*((AG$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AG89-0.5*(AG89-AF89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AH$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AH$4-$G$4:$AQ$4)=0))*((AH$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AH89-0.5*(AH89-AG89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AI$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AI$4-$G$4:$AQ$4)=0))*((AI$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AI89-0.5*(AI89-AH89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AJ$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AJ$4-$G$4:$AQ$4)=0))*((AJ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AJ89-0.5*(AJ89-AI89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AK$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AK$4-$G$4:$AQ$4)=0))*((AK$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AK89-0.5*(AK89-AJ89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AL$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AL$4-$G$4:$AQ$4)=0))*((AL$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AL89-0.5*(AL89-AK89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AM$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AM$4-$G$4:$AQ$4)=0))*((AM$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AM89-0.5*(AM89-AL89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AN$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AN$4-$G$4:$AQ$4)=0))*((AN$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AN89-0.5*(AN89-AM89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AO$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AO$4-$G$4:$AQ$4)=0))*((AO$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AO89-0.5*(AO89-AN89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AP$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AP$4-$G$4:$AQ$4)=0))*((AP$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AP89-0.5*(AP89-AO89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ98" s="39">
         <f>SUMPRODUCT($G$7:$AQ$7*((AQ$4-$G$4:$AQ$4)&gt;=0)*(1-0.5*((AQ$4-$G$4:$AQ$4)=0))*((AQ$4-$G$4:$AQ$4)&lt;Hypothèses!$B$74))+(AQ89-0.5*(AQ89-AP89))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:43" x14ac:dyDescent="0.3">
@@ -15793,11 +15793,11 @@
       </c>
       <c r="E102" s="22">
         <f t="shared" si="39"/>
-        <v>4992000</v>
+        <v>4680000</v>
       </c>
       <c r="F102" s="22">
         <f t="shared" si="40"/>
-        <v>15171000</v>
+        <v>14859000</v>
       </c>
       <c r="G102" s="22">
         <f>0</f>
@@ -15901,51 +15901,51 @@
       </c>
       <c r="AF102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AF98+AF99+AF100+AF101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AG102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AG98+AG99+AG100+AG101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AH102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AH98+AH99+AH100+AH101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AI102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AI98+AI99+AI100+AI101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AJ102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AJ98+AJ99+AJ100+AJ101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AK102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AK98+AK99+AK100+AK101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AL102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AL98+AL99+AL100+AL101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AM102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AM98+AM99+AM100+AM101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AN102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AN98+AN99+AN100+AN101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AO102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AO98+AO99+AO100+AO101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AP102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AP98+AP99+AP100+AP101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
       <c r="AQ102" s="22">
         <f>Hypothèses!$B$103*Hypothèses!$B$47*(AQ98+AQ99+AQ100+AQ101)</f>
-        <v>416000</v>
+        <v>390000</v>
       </c>
     </row>
     <row r="103" spans="1:43" x14ac:dyDescent="0.3">
@@ -17294,11 +17294,11 @@
       </c>
       <c r="E41" s="7">
         <f>Mensuel!E48</f>
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="F41" s="7">
         <f>Mensuel!F48</f>
-        <v>225000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -17344,11 +17344,11 @@
       </c>
       <c r="E43" s="7">
         <f>Mensuel!E50</f>
-        <v>89000</v>
+        <v>0</v>
       </c>
       <c r="F43" s="7">
         <f>Mensuel!F50</f>
-        <v>317000</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -17394,11 +17394,11 @@
       </c>
       <c r="E45" s="9">
         <f>Mensuel!E52</f>
-        <v>164000</v>
+        <v>0</v>
       </c>
       <c r="F45" s="9">
         <f>Mensuel!F52</f>
-        <v>1487000</v>
+        <v>1323000</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -17419,11 +17419,11 @@
       </c>
       <c r="E47" s="11">
         <f>Mensuel!E54</f>
-        <v>10948250</v>
+        <v>10784250</v>
       </c>
       <c r="F47" s="11">
         <f>Mensuel!F54</f>
-        <v>39864611</v>
+        <v>39700611</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -17454,11 +17454,11 @@
       </c>
       <c r="E50" s="7">
         <f>Mensuel!E58</f>
-        <v>1404000</v>
+        <v>624000</v>
       </c>
       <c r="F50" s="7">
         <f>Mensuel!F58</f>
-        <v>4153500</v>
+        <v>3373500</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -17554,11 +17554,11 @@
       </c>
       <c r="E54" s="11">
         <f>Mensuel!E62</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
       <c r="F54" s="11">
         <f>Mensuel!F62</f>
-        <v>46226375</v>
+        <v>45446375</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -17589,11 +17589,11 @@
       </c>
       <c r="E57" s="13">
         <f>Mensuel!E65</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="F57" s="13">
         <f>Mensuel!F65</f>
-        <v>6361764.0000000009</v>
+        <v>5745764.0000000009</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
@@ -17614,7 +17614,7 @@
       </c>
       <c r="E58" s="11">
         <f>Mensuel!E66</f>
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
       <c r="F58" s="11">
         <f>Mensuel!F66</f>
@@ -17828,16 +17828,16 @@
         <v>641142</v>
       </c>
       <c r="D6" s="22">
-        <v>306142</v>
+        <v>-309858</v>
       </c>
       <c r="E6" s="22">
-        <v>-3772083</v>
+        <v>-4030416</v>
       </c>
       <c r="F6" s="22">
-        <v>-208858</v>
+        <v>-467191</v>
       </c>
       <c r="G6" s="22">
-        <v>-543858</v>
+        <v>-643191</v>
       </c>
       <c r="H6" s="22">
         <v>9118334</v>
@@ -17846,7 +17846,7 @@
         <v>9669059</v>
       </c>
       <c r="J6" s="22">
-        <v>9975201</v>
+        <v>9359201</v>
       </c>
       <c r="K6" s="22">
         <v>5845254</v>
@@ -17866,16 +17866,16 @@
         <v>-584347</v>
       </c>
       <c r="D7" s="22">
-        <v>-919347</v>
+        <v>-1426147</v>
       </c>
       <c r="E7" s="22">
-        <v>-5289650</v>
+        <v>-5547983</v>
       </c>
       <c r="F7" s="22">
-        <v>-1434347</v>
+        <v>-1692681</v>
       </c>
       <c r="G7" s="22">
-        <v>-1769347</v>
+        <v>-1759481</v>
       </c>
       <c r="H7" s="22">
         <v>7600767</v>
@@ -17884,10 +17884,10 @@
         <v>6926003</v>
       </c>
       <c r="J7" s="22">
-        <v>6006656</v>
+        <v>5499856</v>
       </c>
       <c r="K7" s="22">
-        <v>5761221</v>
+        <v>5499856</v>
       </c>
       <c r="L7" s="22">
         <v>0</v>
@@ -17904,16 +17904,16 @@
         <v>-1809836</v>
       </c>
       <c r="D8" s="22">
-        <v>-2144836</v>
+        <v>-2542436</v>
       </c>
       <c r="E8" s="22">
-        <v>-6807216</v>
+        <v>-7065550</v>
       </c>
       <c r="F8" s="22">
-        <v>-2659836</v>
+        <v>-2918170</v>
       </c>
       <c r="G8" s="22">
-        <v>-2994836</v>
+        <v>-2875770</v>
       </c>
       <c r="H8" s="22">
         <v>6083200</v>
@@ -17922,10 +17922,10 @@
         <v>4182947</v>
       </c>
       <c r="J8" s="22">
-        <v>2038111</v>
+        <v>1640511</v>
       </c>
       <c r="K8" s="22">
-        <v>2038111</v>
+        <v>1640511</v>
       </c>
       <c r="L8" s="22">
         <v>0</v>
@@ -17942,16 +17942,16 @@
         <v>-3035326</v>
       </c>
       <c r="D9" s="43">
-        <v>-3370326</v>
+        <v>-3658726</v>
       </c>
       <c r="E9" s="43">
-        <v>-8324783</v>
+        <v>-8583116</v>
       </c>
       <c r="F9" s="43">
-        <v>-3885326</v>
+        <v>-4143659</v>
       </c>
       <c r="G9" s="43">
-        <v>-4220326</v>
+        <v>-3992059</v>
       </c>
       <c r="H9" s="43">
         <v>4565634</v>
@@ -17960,10 +17960,10 @@
         <v>1439891</v>
       </c>
       <c r="J9" s="43">
-        <v>-1930434</v>
+        <v>-2218834</v>
       </c>
       <c r="K9" s="43">
-        <v>-1930434</v>
+        <v>-2218834</v>
       </c>
       <c r="L9" s="43">
         <v>10</v>
@@ -17980,16 +17980,16 @@
         <v>-4260815</v>
       </c>
       <c r="D10" s="22">
-        <v>-4595815</v>
+        <v>-4775015</v>
       </c>
       <c r="E10" s="22">
-        <v>-9842350</v>
+        <v>-10100683</v>
       </c>
       <c r="F10" s="22">
-        <v>-5110815</v>
+        <v>-5369148</v>
       </c>
       <c r="G10" s="22">
-        <v>-5445815</v>
+        <v>-5108348</v>
       </c>
       <c r="H10" s="22">
         <v>3048067</v>
@@ -17998,10 +17998,10 @@
         <v>-1303165</v>
       </c>
       <c r="J10" s="22">
-        <v>-5898979</v>
+        <v>-6078179</v>
       </c>
       <c r="K10" s="22">
-        <v>-5898979</v>
+        <v>-6078179</v>
       </c>
       <c r="L10" s="22">
         <v>17</v>
@@ -18018,16 +18018,16 @@
         <v>-5486304</v>
       </c>
       <c r="D11" s="22">
-        <v>-5821304</v>
+        <v>-5891304</v>
       </c>
       <c r="E11" s="22">
-        <v>-11359916</v>
+        <v>-11618250</v>
       </c>
       <c r="F11" s="22">
-        <v>-6336304</v>
+        <v>-6594637</v>
       </c>
       <c r="G11" s="22">
-        <v>-6671304</v>
+        <v>-6224637</v>
       </c>
       <c r="H11" s="22">
         <v>1530500</v>
@@ -18036,10 +18036,10 @@
         <v>-4046220</v>
       </c>
       <c r="J11" s="22">
-        <v>-9867524</v>
+        <v>-9937524</v>
       </c>
       <c r="K11" s="22">
-        <v>-9867524</v>
+        <v>-9937524</v>
       </c>
       <c r="L11" s="22">
         <v>22</v>
@@ -18118,16 +18118,16 @@
         <v>5656950</v>
       </c>
       <c r="D17" s="22">
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E17" s="22">
-        <v>-2129136</v>
+        <v>-2387469</v>
       </c>
       <c r="F17" s="22">
-        <v>4806950</v>
+        <v>4548617</v>
       </c>
       <c r="G17" s="22">
-        <v>2928765</v>
+        <v>2859232</v>
       </c>
       <c r="H17" s="22">
         <v>10761281</v>
@@ -18136,7 +18136,7 @@
         <v>16327814</v>
       </c>
       <c r="J17" s="22">
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
       <c r="K17" s="22">
         <v>5845254</v>
@@ -18156,16 +18156,16 @@
         <v>3559530</v>
       </c>
       <c r="D18" s="22">
-        <v>2936530</v>
+        <v>2429730</v>
       </c>
       <c r="E18" s="22">
-        <v>-3995817</v>
+        <v>-4254150</v>
       </c>
       <c r="F18" s="22">
-        <v>2709530</v>
+        <v>2451197</v>
       </c>
       <c r="G18" s="22">
-        <v>1846457</v>
+        <v>2008364</v>
       </c>
       <c r="H18" s="22">
         <v>8894600</v>
@@ -18174,7 +18174,7 @@
         <v>12363713</v>
       </c>
       <c r="J18" s="22">
-        <v>15300243</v>
+        <v>14793443</v>
       </c>
       <c r="K18" s="22">
         <v>5785672</v>
@@ -18194,16 +18194,16 @@
         <v>1462110</v>
       </c>
       <c r="D19" s="22">
-        <v>839110</v>
+        <v>441510</v>
       </c>
       <c r="E19" s="22">
-        <v>-5824893</v>
+        <v>-6083227</v>
       </c>
       <c r="F19" s="22">
-        <v>612110</v>
+        <v>353777</v>
       </c>
       <c r="G19" s="22">
-        <v>-10890</v>
+        <v>108177</v>
       </c>
       <c r="H19" s="22">
         <v>7065523</v>
@@ -18212,7 +18212,7 @@
         <v>8437217</v>
       </c>
       <c r="J19" s="22">
-        <v>9276327</v>
+        <v>8878727</v>
       </c>
       <c r="K19" s="22">
         <v>5647838</v>
@@ -18232,16 +18232,16 @@
         <v>-556848</v>
       </c>
       <c r="D20" s="43">
-        <v>-1179848</v>
+        <v>-1468248</v>
       </c>
       <c r="E20" s="43">
-        <v>-7601564</v>
+        <v>-7859897</v>
       </c>
       <c r="F20" s="43">
-        <v>-1406848</v>
+        <v>-1665181</v>
       </c>
       <c r="G20" s="43">
-        <v>-2029848</v>
+        <v>-1801581</v>
       </c>
       <c r="H20" s="43">
         <v>5288853</v>
@@ -18250,10 +18250,10 @@
         <v>4641588</v>
       </c>
       <c r="J20" s="43">
-        <v>3461740</v>
+        <v>3173340</v>
       </c>
       <c r="K20" s="43">
-        <v>3424664</v>
+        <v>3173340</v>
       </c>
       <c r="L20" s="43">
         <v>0</v>
@@ -18270,16 +18270,16 @@
         <v>-2408334</v>
       </c>
       <c r="D21" s="22">
-        <v>-3031334</v>
+        <v>-3210534</v>
       </c>
       <c r="E21" s="22">
-        <v>-9350323</v>
+        <v>-9608656</v>
       </c>
       <c r="F21" s="22">
-        <v>-3258334</v>
+        <v>-3516667</v>
       </c>
       <c r="G21" s="22">
-        <v>-3881334</v>
+        <v>-3543867</v>
       </c>
       <c r="H21" s="22">
         <v>3540094</v>
@@ -18288,13 +18288,13 @@
         <v>1041343</v>
       </c>
       <c r="J21" s="22">
-        <v>-1989991</v>
+        <v>-2169191</v>
       </c>
       <c r="K21" s="22">
-        <v>-1989991</v>
+        <v>-2169191</v>
       </c>
       <c r="L21" s="22">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
@@ -18308,16 +18308,16 @@
         <v>-4259820</v>
       </c>
       <c r="D22" s="22">
-        <v>-4882820</v>
+        <v>-4952820</v>
       </c>
       <c r="E22" s="22">
-        <v>-11099082</v>
+        <v>-11357415</v>
       </c>
       <c r="F22" s="22">
-        <v>-5109820</v>
+        <v>-5368153</v>
       </c>
       <c r="G22" s="22">
-        <v>-5732820</v>
+        <v>-5286153</v>
       </c>
       <c r="H22" s="22">
         <v>1791335</v>
@@ -18326,10 +18326,10 @@
         <v>-2558902</v>
       </c>
       <c r="J22" s="22">
-        <v>-7441722</v>
+        <v>-7511722</v>
       </c>
       <c r="K22" s="22">
-        <v>-7441722</v>
+        <v>-7511722</v>
       </c>
       <c r="L22" s="22">
         <v>21</v>
@@ -18587,10 +18587,10 @@
         <v>5656950</v>
       </c>
       <c r="E45" s="22">
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="F45" s="22">
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
       <c r="G45" s="22">
         <v>5845254</v>
@@ -18613,13 +18613,13 @@
         <v>-556848</v>
       </c>
       <c r="E46" s="22">
-        <v>-1179848</v>
+        <v>-1468248</v>
       </c>
       <c r="F46" s="22">
-        <v>3461740</v>
+        <v>3173340</v>
       </c>
       <c r="G46" s="22">
-        <v>3424664</v>
+        <v>3173340</v>
       </c>
       <c r="H46" s="46" t="s">
         <v>71</v>
@@ -18639,10 +18639,10 @@
         <v>4954950</v>
       </c>
       <c r="E47" s="22">
-        <v>4331950</v>
+        <v>3715950</v>
       </c>
       <c r="F47" s="22">
-        <v>19689333</v>
+        <v>19073333</v>
       </c>
       <c r="G47" s="22">
         <v>5845254</v>
@@ -18665,13 +18665,13 @@
         <v>-989280</v>
       </c>
       <c r="E48" s="22">
-        <v>-1612280</v>
+        <v>-1900680</v>
       </c>
       <c r="F48" s="22">
-        <v>2437171</v>
+        <v>2148771</v>
       </c>
       <c r="G48" s="22">
-        <v>2437171</v>
+        <v>2148771</v>
       </c>
       <c r="H48" s="46" t="s">
         <v>71</v>
@@ -18691,10 +18691,10 @@
         <v>9130350</v>
       </c>
       <c r="E49" s="22">
-        <v>8315350</v>
+        <v>7699350</v>
       </c>
       <c r="F49" s="22">
-        <v>29282023</v>
+        <v>28666023</v>
       </c>
       <c r="G49" s="22">
         <v>5845254</v>
@@ -18717,10 +18717,10 @@
         <v>1415370</v>
       </c>
       <c r="E50" s="22">
-        <v>600370</v>
+        <v>311970</v>
       </c>
       <c r="F50" s="22">
-        <v>7743100</v>
+        <v>7454700</v>
       </c>
       <c r="G50" s="22">
         <v>4939723</v>
@@ -18743,10 +18743,10 @@
         <v>4438300</v>
       </c>
       <c r="E51" s="22">
-        <v>4153300</v>
+        <v>3537300</v>
       </c>
       <c r="F51" s="22">
-        <v>18637688</v>
+        <v>18021688</v>
       </c>
       <c r="G51" s="22">
         <v>5845254</v>
@@ -18769,13 +18769,13 @@
         <v>-2431940</v>
       </c>
       <c r="E52" s="22">
-        <v>-2716940</v>
+        <v>-3005340</v>
       </c>
       <c r="F52" s="22">
-        <v>-844129</v>
+        <v>-1132529</v>
       </c>
       <c r="G52" s="22">
-        <v>-844129</v>
+        <v>-1132529</v>
       </c>
       <c r="H52" s="46" t="s">
         <v>71</v>
@@ -19709,7 +19709,7 @@
         <v>235</v>
       </c>
       <c r="B74" s="17">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>236</v>
@@ -20432,11 +20432,11 @@
       </c>
       <c r="D5" s="22">
         <f>Mensuel!E58</f>
-        <v>1404000</v>
+        <v>624000</v>
       </c>
       <c r="E5" s="22">
         <f>SUM(B5:D5)</f>
-        <v>4153500</v>
+        <v>3373500</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -20516,11 +20516,11 @@
       </c>
       <c r="D9" s="24">
         <f>SUM(D5:D8)</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
       <c r="E9" s="24">
         <f>SUM(E5:E8)</f>
-        <v>46226375</v>
+        <v>45446375</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -20533,7 +20533,7 @@
       </c>
       <c r="D10" s="36">
         <f>IF(C9=0,0,D9/C9-1)</f>
-        <v>0</v>
+        <v>-4.880429477794046E-2</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -20550,7 +20550,7 @@
       </c>
       <c r="D11" s="22">
         <f>D9/12</f>
-        <v>1331850</v>
+        <v>1266850</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -20698,11 +20698,11 @@
       </c>
       <c r="D20" s="36">
         <f>IF(D19=0,0,D9/D19)</f>
-        <v>0.19495718363463369</v>
+        <v>0.18544243577545194</v>
       </c>
       <c r="E20" s="36">
         <f>IF(E19=0,0,E9/E19)</f>
-        <v>0.20461404785812312</v>
+        <v>0.20116149599072414</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
@@ -20719,11 +20719,11 @@
       </c>
       <c r="D21" s="36">
         <f>IF(D9=0,0,(D7+D8)/D9)</f>
-        <v>0.79795021961932655</v>
+        <v>0.83889173935351458</v>
       </c>
       <c r="E21" s="36">
         <f>IF(E9=0,0,(E7+E8)/E9)</f>
-        <v>0.75000527296375719</v>
+        <v>0.7628776772624879</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
@@ -21991,11 +21991,11 @@
       </c>
       <c r="E41" s="22">
         <f>Mensuel!E48</f>
-        <v>75000</v>
+        <v>0</v>
       </c>
       <c r="F41" s="22">
         <f>Mensuel!F48</f>
-        <v>225000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -22043,11 +22043,11 @@
       </c>
       <c r="E43" s="22">
         <f>Mensuel!E50</f>
-        <v>89000</v>
+        <v>0</v>
       </c>
       <c r="F43" s="22">
         <f>Mensuel!F50</f>
-        <v>317000</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
@@ -22094,11 +22094,11 @@
       </c>
       <c r="E45" s="24">
         <f>Mensuel!E52</f>
-        <v>164000</v>
+        <v>0</v>
       </c>
       <c r="F45" s="24">
         <f>Mensuel!F52</f>
-        <v>1487000</v>
+        <v>1323000</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -22119,11 +22119,11 @@
       </c>
       <c r="E47" s="24">
         <f>Mensuel!E54</f>
-        <v>10948250</v>
+        <v>10784250</v>
       </c>
       <c r="F47" s="24">
         <f>Mensuel!F54</f>
-        <v>39864611</v>
+        <v>39700611</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
@@ -22171,19 +22171,19 @@
       </c>
       <c r="C51" s="22">
         <f>Mensuel!C70</f>
-        <v>516666.66666666669</v>
+        <v>775000.00000000012</v>
       </c>
       <c r="D51" s="22">
         <f>Mensuel!D70</f>
-        <v>516666.66666666669</v>
+        <v>775000.00000000012</v>
       </c>
       <c r="E51" s="22">
         <f>Mensuel!E70</f>
-        <v>516666.66666666669</v>
+        <v>0</v>
       </c>
       <c r="F51" s="22">
         <f>Mensuel!F70</f>
-        <v>1550000</v>
+        <v>1550000.0000000002</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -22407,7 +22407,7 @@
       </c>
       <c r="C7" s="22">
         <f>-Mensuel!C70</f>
-        <v>-516666.66666666669</v>
+        <v>-775000.00000000012</v>
       </c>
       <c r="D7" s="22">
         <v>0</v>
@@ -22417,7 +22417,7 @@
       </c>
       <c r="F7" s="22">
         <f>SUM(B7:E7)</f>
-        <v>-2891666.6666666665</v>
+        <v>-3150000</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -22501,7 +22501,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(C6:C10)</f>
-        <v>531101.35670502495</v>
+        <v>272768.02337169158</v>
       </c>
       <c r="D11" s="24">
         <f>SUM(D6:D10)</f>
@@ -22513,7 +22513,7 @@
       </c>
       <c r="F11" s="24">
         <f>SUM(F6:F10)</f>
-        <v>8476072.333333334</v>
+        <v>8217739</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -22526,7 +22526,7 @@
       </c>
       <c r="C12" s="36">
         <f>IF(C6=0,0,C11/C6)</f>
-        <v>0.3947241595726681</v>
+        <v>0.2027261414876935</v>
       </c>
       <c r="D12" s="36">
         <f>IF(D6=0,0,D11/D6)</f>
@@ -22538,7 +22538,7 @@
       </c>
       <c r="F12" s="36">
         <f>IF(F6=0,0,F11/F6)</f>
-        <v>0.59431266240007674</v>
+        <v>0.57619922906890531</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -22576,7 +22576,7 @@
       </c>
       <c r="C14" s="24">
         <f>C11+C13</f>
-        <v>-150223.13113764767</v>
+        <v>-408556.46447098104</v>
       </c>
       <c r="D14" s="24">
         <f>D11+D13</f>
@@ -22588,7 +22588,7 @@
       </c>
       <c r="F14" s="24">
         <f>F11+F13</f>
-        <v>1254197.333333334</v>
+        <v>995864</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -22626,7 +22626,7 @@
       </c>
       <c r="C16" s="22">
         <f>IF(C15=0,0,C11/(C15*Hypothèses!$B$47*12))</f>
-        <v>1702.2479381571313</v>
+        <v>874.2564851656781</v>
       </c>
       <c r="D16" s="22">
         <f>IF(D15=0,0,D11/(D15*Hypothèses!$B$47*12))</f>
@@ -22638,7 +22638,7 @@
       </c>
       <c r="F16" s="22">
         <f>IF(F15=0,0,F11/(F15*Hypothèses!$B$47*12))</f>
-        <v>1552.3942002442004</v>
+        <v>1505.0804029304029</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -22651,7 +22651,7 @@
       </c>
       <c r="C17" s="22">
         <f>IF(C15=0,0,C14/(C15*Hypothèses!$B$47*12))</f>
-        <v>-481.48439467194765</v>
+        <v>-1309.4758476634008</v>
       </c>
       <c r="D17" s="22">
         <f>IF(D15=0,0,D14/(D15*Hypothèses!$B$47*12))</f>
@@ -22663,7 +22663,7 @@
       </c>
       <c r="F17" s="22">
         <f>IF(F15=0,0,F14/(F15*Hypothèses!$B$47*12))</f>
-        <v>229.70647130647143</v>
+        <v>182.39267399267399</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -22731,7 +22731,7 @@
       </c>
       <c r="C22" s="22">
         <f>-Mensuel!D70</f>
-        <v>-516666.66666666669</v>
+        <v>-775000.00000000012</v>
       </c>
       <c r="D22" s="22">
         <v>0</v>
@@ -22741,7 +22741,7 @@
       </c>
       <c r="F22" s="22">
         <f>SUM(B22:E22)</f>
-        <v>-516666.66666666669</v>
+        <v>-775000.00000000012</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -22825,7 +22825,7 @@
       </c>
       <c r="C26" s="24">
         <f>SUM(C21:C25)</f>
-        <v>654827.14874722483</v>
+        <v>396493.8154138914</v>
       </c>
       <c r="D26" s="24">
         <f>SUM(D21:D25)</f>
@@ -22837,7 +22837,7 @@
       </c>
       <c r="F26" s="24">
         <f>SUM(F21:F25)</f>
-        <v>13501533.333333334</v>
+        <v>13243200</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -22850,7 +22850,7 @@
       </c>
       <c r="C27" s="36">
         <f>IF(C21=0,0,C26/C21)</f>
-        <v>0.466401103096314</v>
+        <v>0.28240300243154659</v>
       </c>
       <c r="D27" s="36">
         <f>IF(D21=0,0,D26/D21)</f>
@@ -22862,7 +22862,7 @@
       </c>
       <c r="F27" s="36">
         <f>IF(F21=0,0,F26/F21)</f>
-        <v>0.84478565737716549</v>
+        <v>0.82862184179900134</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -22900,7 +22900,7 @@
       </c>
       <c r="C29" s="24">
         <f>C26+C28</f>
-        <v>-79689.688734473544</v>
+        <v>-338023.02206780697</v>
       </c>
       <c r="D29" s="24">
         <f>D26+D28</f>
@@ -22912,7 +22912,7 @@
       </c>
       <c r="F29" s="24">
         <f>F26+F28</f>
-        <v>5140283.333333333</v>
+        <v>4881949.9999999991</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -22950,7 +22950,7 @@
       </c>
       <c r="C31" s="22">
         <f>IF(C30=0,0,C26/(C30*Hypothèses!$B$47*12))</f>
-        <v>2098.8049639334131</v>
+        <v>1270.8135109419595</v>
       </c>
       <c r="D31" s="22">
         <f>IF(D30=0,0,D26/(D30*Hypothèses!$B$47*12))</f>
@@ -22962,7 +22962,7 @@
       </c>
       <c r="F31" s="22">
         <f>IF(F30=0,0,F26/(F30*Hypothèses!$B$47*12))</f>
-        <v>2060.6735856735859</v>
+        <v>2021.2454212454213</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
@@ -22975,7 +22975,7 @@
       </c>
       <c r="C32" s="22">
         <f>IF(C30=0,0,C29/(C30*Hypothèses!$B$47*12))</f>
-        <v>-255.41566902074854</v>
+        <v>-1083.4071220122019</v>
       </c>
       <c r="D32" s="22">
         <f>IF(D30=0,0,D29/(D30*Hypothèses!$B$47*12))</f>
@@ -22987,7 +22987,7 @@
       </c>
       <c r="F32" s="22">
         <f>IF(F30=0,0,F29/(F30*Hypothèses!$B$47*12))</f>
-        <v>784.53652828652821</v>
+        <v>745.10836385836376</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
@@ -23030,7 +23030,7 @@
       </c>
       <c r="C36" s="22">
         <f>Mensuel!E58</f>
-        <v>1404000</v>
+        <v>624000</v>
       </c>
       <c r="D36" s="22">
         <f>Mensuel!E60</f>
@@ -23042,7 +23042,7 @@
       </c>
       <c r="F36" s="25">
         <f>SUM(B36:E36)</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
@@ -23055,7 +23055,7 @@
       </c>
       <c r="C37" s="22">
         <f>-Mensuel!E70</f>
-        <v>-516666.66666666669</v>
+        <v>0</v>
       </c>
       <c r="D37" s="22">
         <v>0</v>
@@ -23065,7 +23065,7 @@
       </c>
       <c r="F37" s="22">
         <f>SUM(B37:E37)</f>
-        <v>-516666.66666666669</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
@@ -23078,7 +23078,7 @@
       </c>
       <c r="C38" s="22">
         <f>-Mensuel!E48</f>
-        <v>-75000</v>
+        <v>0</v>
       </c>
       <c r="D38" s="22">
         <v>0</v>
@@ -23088,7 +23088,7 @@
       </c>
       <c r="F38" s="22">
         <f>SUM(B38:E38)</f>
-        <v>-75000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -23101,7 +23101,7 @@
       </c>
       <c r="C39" s="22">
         <f>-Mensuel!E50</f>
-        <v>-89000</v>
+        <v>0</v>
       </c>
       <c r="D39" s="22">
         <v>0</v>
@@ -23111,7 +23111,7 @@
       </c>
       <c r="F39" s="22">
         <f>SUM(B39:E39)</f>
-        <v>-89000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -23149,7 +23149,7 @@
       </c>
       <c r="C41" s="24">
         <f>SUM(C36:C40)</f>
-        <v>654827.14874722483</v>
+        <v>555493.81541389157</v>
       </c>
       <c r="D41" s="24">
         <f>SUM(D36:D40)</f>
@@ -23161,7 +23161,7 @@
       </c>
       <c r="F41" s="24">
         <f>SUM(F36:F40)</f>
-        <v>13501533.333333334</v>
+        <v>13402200</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
@@ -23174,7 +23174,7 @@
       </c>
       <c r="C42" s="36">
         <f>IF(C36=0,0,C41/C36)</f>
-        <v>0.466401103096314</v>
+        <v>0.89021444777867242</v>
       </c>
       <c r="D42" s="36">
         <f>IF(D36=0,0,D41/D36)</f>
@@ -23186,7 +23186,7 @@
       </c>
       <c r="F42" s="36">
         <f>IF(F36=0,0,F41/F36)</f>
-        <v>0.84478565737716549</v>
+        <v>0.8815960847772033</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
@@ -23195,19 +23195,19 @@
       </c>
       <c r="B43" s="22">
         <f>-(Mensuel!E39-Mensuel!E33)*IF($F36=0,0,B36/$F36)</f>
-        <v>-1026019.765739385</v>
+        <v>-1078663.160595177</v>
       </c>
       <c r="C43" s="22">
         <f>-(Mensuel!E39-Mensuel!E33)*IF($F36=0,0,C36/$F36)</f>
-        <v>-789245.97364568082</v>
+        <v>-368773.7301180092</v>
       </c>
       <c r="D43" s="22">
         <f>-(Mensuel!E39-Mensuel!E33)*IF($F36=0,0,D36/$F36)</f>
-        <v>-3827842.9721815516</v>
+        <v>-4024243.3299127757</v>
       </c>
       <c r="E43" s="22">
         <f>-(Mensuel!E39-Mensuel!E33)*IF($F36=0,0,E36/$F36)</f>
-        <v>-3341141.2884333823</v>
+        <v>-3512569.7793740379</v>
       </c>
       <c r="F43" s="22">
         <f>SUM(B43:E43)</f>
@@ -23220,23 +23220,23 @@
       </c>
       <c r="B44" s="24">
         <f>B41+B43</f>
-        <v>598799.64434624766</v>
+        <v>546156.24949045572</v>
       </c>
       <c r="C44" s="24">
         <f>C41+C43</f>
-        <v>-134418.82489845599</v>
+        <v>186720.08529588237</v>
       </c>
       <c r="D44" s="24">
         <f>D41+D43</f>
-        <v>2136875.7718717312</v>
+        <v>1940475.4141405071</v>
       </c>
       <c r="E44" s="24">
         <f>E41+E43</f>
-        <v>1916026.7420138111</v>
+        <v>1744598.2510731556</v>
       </c>
       <c r="F44" s="24">
         <f>F41+F43</f>
-        <v>4517283.333333334</v>
+        <v>4417950</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -23274,7 +23274,7 @@
       </c>
       <c r="C46" s="22">
         <f>IF(C45=0,0,C41/(C45*Hypothèses!$B$47*12))</f>
-        <v>2098.8049639334131</v>
+        <v>1780.4288955573447</v>
       </c>
       <c r="D46" s="22">
         <f>IF(D45=0,0,D41/(D45*Hypothèses!$B$47*12))</f>
@@ -23286,7 +23286,7 @@
       </c>
       <c r="F46" s="22">
         <f>IF(F45=0,0,F41/(F45*Hypothèses!$B$47*12))</f>
-        <v>2060.6735856735859</v>
+        <v>2045.5128205128206</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -23295,23 +23295,23 @@
       </c>
       <c r="B47" s="22">
         <f>IF(B45=0,0,B44/(B45*Hypothèses!$B$47*12))</f>
-        <v>383.84592586297924</v>
+        <v>350.10015992977929</v>
       </c>
       <c r="C47" s="22">
         <f>IF(C45=0,0,C44/(C45*Hypothèses!$B$47*12))</f>
-        <v>-430.82956698223074</v>
+        <v>598.46181184577677</v>
       </c>
       <c r="D47" s="22">
         <f>IF(D45=0,0,D44/(D45*Hypothèses!$B$47*12))</f>
-        <v>760.99564525346545</v>
+        <v>691.05249791328606</v>
       </c>
       <c r="E47" s="22">
         <f>IF(E45=0,0,E44/(E45*Hypothèses!$B$47*12))</f>
-        <v>1023.5185587680616</v>
+        <v>931.94351018865143</v>
       </c>
       <c r="F47" s="22">
         <f>IF(F45=0,0,F44/(F45*Hypothèses!$B$47*12))</f>
-        <v>689.45105820105834</v>
+        <v>674.29029304029302</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -23342,15 +23342,15 @@
       </c>
       <c r="B51" s="22">
         <f>F14</f>
-        <v>1254197.333333334</v>
+        <v>995864</v>
       </c>
       <c r="C51" s="22">
         <f>F29</f>
-        <v>5140283.333333333</v>
+        <v>4881949.9999999991</v>
       </c>
       <c r="D51" s="22">
         <f>F44</f>
-        <v>4517283.333333334</v>
+        <v>4417950</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -23393,15 +23393,15 @@
       </c>
       <c r="B54" s="25">
         <f>SUM(B51:B53)</f>
-        <v>-2129135.9999999991</v>
+        <v>-2387469.333333333</v>
       </c>
       <c r="C54" s="25">
         <f>SUM(C51:C53)</f>
-        <v>4806950</v>
+        <v>4548616.666666666</v>
       </c>
       <c r="D54" s="25">
         <f>SUM(D51:D53)</f>
-        <v>4183950.0000000009</v>
+        <v>4084616.666666667</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -23410,15 +23410,15 @@
       </c>
       <c r="B55" s="22">
         <f>Résultat!B12</f>
-        <v>-2129136</v>
+        <v>-2387469.333333334</v>
       </c>
       <c r="C55" s="22">
         <f>Résultat!C12</f>
-        <v>4806950</v>
+        <v>4548616.666666667</v>
       </c>
       <c r="D55" s="22">
         <f>Résultat!D12</f>
-        <v>4183950</v>
+        <v>4084616.666666667</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -23502,11 +23502,11 @@
       </c>
       <c r="D6" s="25">
         <f>Mensuel!E62</f>
-        <v>15982200</v>
+        <v>15202200</v>
       </c>
       <c r="E6" s="25">
         <f t="shared" ref="E6:E14" si="0">SUM(B6:D6)</f>
-        <v>46226375</v>
+        <v>45446375</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -23544,11 +23544,11 @@
       </c>
       <c r="D8" s="22">
         <f>-Mensuel!E52</f>
-        <v>-164000</v>
+        <v>0</v>
       </c>
       <c r="E8" s="22">
         <f t="shared" si="0"/>
-        <v>-1487000</v>
+        <v>-1323000</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -23565,11 +23565,11 @@
       </c>
       <c r="D9" s="24">
         <f>D6+D7+D8</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E9" s="24">
         <f t="shared" si="0"/>
-        <v>14836764</v>
+        <v>14220764</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -23578,15 +23578,15 @@
       </c>
       <c r="B10" s="22">
         <f>-Mensuel!C73</f>
-        <v>-3225000</v>
+        <v>-3483333.333333334</v>
       </c>
       <c r="C10" s="22">
         <f>-Mensuel!D73</f>
-        <v>-850000.00000000012</v>
+        <v>-1108333.3333333333</v>
       </c>
       <c r="D10" s="22">
         <f>-Mensuel!E73</f>
-        <v>-850000.00000000012</v>
+        <v>-333333.33333333326</v>
       </c>
       <c r="E10" s="22">
         <f t="shared" si="0"/>
@@ -23620,19 +23620,19 @@
       </c>
       <c r="B12" s="24">
         <f>B9+B10+B11</f>
-        <v>-2129136</v>
+        <v>-2387469.333333334</v>
       </c>
       <c r="C12" s="24">
         <f>C9+C10+C11</f>
-        <v>4806950</v>
+        <v>4548616.666666667</v>
       </c>
       <c r="D12" s="24">
         <f>D9+D10+D11</f>
-        <v>4183950</v>
+        <v>4084616.666666667</v>
       </c>
       <c r="E12" s="24">
         <f t="shared" si="0"/>
-        <v>6861764</v>
+        <v>6245764</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -23649,11 +23649,11 @@
       </c>
       <c r="D13" s="22">
         <f>-IF(3&lt;=Hypothèses!$B$89,0,Hypothèses!$B$88*MAX(0,D12+MIN(0,B12+C12)))</f>
-        <v>-1255185</v>
+        <v>-1225385</v>
       </c>
       <c r="E13" s="22">
         <f t="shared" si="0"/>
-        <v>-1255185</v>
+        <v>-1225385</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -23662,19 +23662,19 @@
       </c>
       <c r="B14" s="24">
         <f>B12+B13</f>
-        <v>-2129136</v>
+        <v>-2387469.333333334</v>
       </c>
       <c r="C14" s="24">
         <f>C12+C13</f>
-        <v>4806950</v>
+        <v>4548616.666666667</v>
       </c>
       <c r="D14" s="24">
         <f>D12+D13</f>
-        <v>2928765</v>
+        <v>2859231.666666667</v>
       </c>
       <c r="E14" s="24">
         <f t="shared" si="0"/>
-        <v>5606579</v>
+        <v>5020379</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -23734,19 +23734,19 @@
       </c>
       <c r="B19" s="24">
         <f>B14+B17+B18</f>
-        <v>-2824136</v>
+        <v>-3082469.333333334</v>
       </c>
       <c r="C19" s="24">
         <f>C14+C17+C18</f>
-        <v>4016950</v>
+        <v>3758616.666666667</v>
       </c>
       <c r="D19" s="24">
         <f>D14+D17+D18</f>
-        <v>2138765</v>
+        <v>2069231.666666667</v>
       </c>
       <c r="E19" s="24">
         <f>SUM(B19:D19)</f>
-        <v>3331579</v>
+        <v>2745379</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -23755,15 +23755,15 @@
       </c>
       <c r="B20" s="22">
         <f>B19</f>
-        <v>-2824136</v>
+        <v>-3082469.333333334</v>
       </c>
       <c r="C20" s="22">
         <f>B20+C19</f>
-        <v>1192814</v>
+        <v>676147.33333333302</v>
       </c>
       <c r="D20" s="22">
         <f>C20+D19</f>
-        <v>3331579</v>
+        <v>2745379</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -23772,19 +23772,19 @@
       </c>
       <c r="B21" s="36">
         <f>IF(B6=0,0,B19/B6)</f>
-        <v>-0.19801857737094616</v>
+        <v>-0.21613201070211763</v>
       </c>
       <c r="C21" s="36">
         <f>IF(C6=0,0,C19/C6)</f>
-        <v>0.25133898962595885</v>
+        <v>0.23517517404779487</v>
       </c>
       <c r="D21" s="36">
         <f>IF(D6=0,0,D19/D6)</f>
-        <v>0.13382168912915618</v>
+        <v>0.13611396157573685</v>
       </c>
       <c r="E21" s="36">
         <f>IF(E6=0,0,E19/E6)</f>
-        <v>7.2070955163583555E-2</v>
+        <v>6.0409196553080413E-2</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -23802,19 +23802,19 @@
       </c>
       <c r="B24" s="22">
         <f>B14</f>
-        <v>-2129136</v>
+        <v>-2387469.333333334</v>
       </c>
       <c r="C24" s="22">
         <f>C14</f>
-        <v>4806950</v>
+        <v>4548616.666666667</v>
       </c>
       <c r="D24" s="22">
         <f>D14</f>
-        <v>2928765</v>
+        <v>2859231.666666667</v>
       </c>
       <c r="E24" s="22">
         <f t="shared" ref="E24:E32" si="1">SUM(B24:D24)</f>
-        <v>5606579</v>
+        <v>5020379</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -23823,15 +23823,15 @@
       </c>
       <c r="B25" s="22">
         <f>-B10</f>
-        <v>3225000</v>
+        <v>3483333.333333334</v>
       </c>
       <c r="C25" s="22">
         <f>-C10</f>
-        <v>850000.00000000012</v>
+        <v>1108333.3333333333</v>
       </c>
       <c r="D25" s="22">
         <f>-D10</f>
-        <v>850000.00000000012</v>
+        <v>333333.33333333326</v>
       </c>
       <c r="E25" s="22">
         <f t="shared" si="1"/>
@@ -23852,11 +23852,11 @@
       </c>
       <c r="D26" s="22">
         <f>-D13</f>
-        <v>1255185</v>
+        <v>1225385</v>
       </c>
       <c r="E26" s="22">
         <f t="shared" si="1"/>
-        <v>1255185</v>
+        <v>1225385</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -23936,11 +23936,11 @@
       </c>
       <c r="D30" s="24">
         <f>SUM(D24:D29)</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E30" s="24">
         <f t="shared" si="1"/>
-        <v>6361764.0000000009</v>
+        <v>5745764.0000000009</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -23957,11 +23957,11 @@
       </c>
       <c r="D31" s="22">
         <f>Mensuel!E65</f>
-        <v>5033950</v>
+        <v>4417950</v>
       </c>
       <c r="E31" s="22">
         <f t="shared" si="1"/>
-        <v>6361764.0000000009</v>
+        <v>5745764.0000000009</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="D33" s="25">
         <f>Mensuel!E66</f>
-        <v>21361764</v>
+        <v>20745764</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Marketing de lancement : spots video par IA (Higgsfield) integres a l'enveloppe de 1 M (pilote Plus 39 200 F, Ultra 309 600 F au plus), dollar a 800 F dans le plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TamCar_resultat_complet_v2.xlsx
+++ b/TamCar_resultat_complet_v2.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="535">
   <si>
     <t>TamCar — Résultat complet : démarrage, recettes, charges, marge, résultat (FCFA)</t>
   </si>
@@ -1631,6 +1631,9 @@
   </si>
   <si>
     <t>Années 2 et 3 : les motos sont cédées aux conducteurs à 12 mois (plus d'assurance ni de tracker payés par TamCar) ; les tricycles restent à TamCar 36 mois.</t>
+  </si>
+  <si>
+    <t>Comprend la création de spots vidéo par IA (Higgsfield) : pilote 39 200 F (forfait Plus, 49 $, 1 mois), puis 309 600 F au plus (forfait Ultra, 3 × 129 $) si le pilote convainc, dollar à 800 F ; le solde couvre la photo et le sponsoring ; la diffusion payante n'est pas budgétée</t>
   </si>
 </sst>
 </file>
@@ -19257,7 +19260,7 @@
         <v>1000000</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>159</v>
+        <v>534</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>